<commit_message>
PAUSED (task175): stage 4 round 1 fixes, waiting on round 2 readers
The estimand is filed as the expected number of distinct lots, and the call is the three areas' total
at the nearest 50: 300 (293.2), with an honest family of 283.2 to 315.6 inside the bin and the
per-area figures dropped. The ask primaries are re-sited: meter re-sets logged as fresh installs, and
receipt numbers that run by drawer and day. All 24 ask figures miss on the cracker's route and on
both round 1 readers' routes. The plat index is recorded in order. Every stage 3 gate re-run green.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task175/golden/uep_2027_permit_forecast.xlsx
+++ b/task175/golden/uep_2027_permit_forecast.xlsx
@@ -44,9 +44,6 @@
     <t>On streets with no home standing</t>
   </si>
   <si>
-    <t>Permits forecast, 2027</t>
-  </si>
-  <si>
     <t>North 6</t>
   </si>
   <si>
@@ -68,7 +65,10 @@
     <t>Three areas</t>
   </si>
   <si>
-    <t>Area figures to the nearest 5 and the total to the nearest 10, the total rounded from the unrounded sum. Each vacant lot's 2027 chance of a permit is taken from served vacant lots 2008 to 2026 with as many homes standing on their street (both sides of the hundred-block) on 1 January, canal lots apart, at the 2026 level; Northwest 3 lots count at the well and septic rate until its lines are accepted.</t>
+    <t>Single-family permits forecast for 2027, the three areas together (nearest 50)</t>
+  </si>
+  <si>
+    <t>The forecast is the expected number of distinct lots permitted in 2027. Each vacant lot's 2027 chance of a permit is taken from served vacant lots 2008 to 2026 with as many homes standing on their street (both sides of the hundred-block) on 1 January, canal lots apart, at the 2026 level; Northwest 3 lots count at the well and septic rate until its lines are accepted.</t>
   </si>
   <si>
     <t>Source: Calusa County Property Appraiser 2026 roll; Building Division permits 2008 to 2026; program schedule Revision 12.</t>
@@ -77,7 +77,7 @@
     <t>New single-family connections, fiscal 2026</t>
   </si>
   <si>
-    <t>Meters installed at premises with no account opened before the install; quarter of the install date.</t>
+    <t>A premise's first meter install, at a premise with no account opened before it; quarter of the install date.</t>
   </si>
   <si>
     <t>Phase</t>
@@ -116,13 +116,13 @@
     <t>All served areas</t>
   </si>
   <si>
-    <t>AMI head-end installs at premises already billed before the install are meter exchanges, not connections. Phases as the program schedule groups the areas; premises are placed by parcel or service address.</t>
+    <t>AMI head-end installs at premises already billed before the install are meter exchanges, and a second install at a premise is a meter set again, not connections. Phases as the program schedule groups the areas; premises are placed by parcel or service address.</t>
   </si>
   <si>
     <t>Water and sewer capacity fees received, fiscal 2026</t>
   </si>
   <si>
-    <t>Cashiering receipts, fee code CAPWS, by receipt date; each receipt counted once.</t>
+    <t>Cashiering receipts, fee code CAPWS, by receipt date; each payment (receipt number and payer) counted once.</t>
   </si>
   <si>
     <t>Quarter</t>
@@ -131,7 +131,7 @@
     <t>Fees received (USD)</t>
   </si>
   <si>
-    <t>A builder's receipt covering several permits carries the receipt amount on each permit line.</t>
+    <t>A builder's receipt covering several permits carries the receipt amount on each permit line; receipt numbers run by drawer and day.</t>
   </si>
 </sst>
 </file>
@@ -207,7 +207,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -219,6 +219,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
@@ -523,7 +525,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26F8B19F-76A7-53F0-AAEA-A8C6A518E90D}">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.7109375" customWidth="1"/>
@@ -531,20 +533,19 @@
     <col min="3" max="3" width="14.7109375" customWidth="1"/>
     <col min="4" max="4" width="14.7109375" customWidth="1"/>
     <col min="5" max="5" width="17.7109375" customWidth="1"/>
-    <col min="6" max="6" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -560,16 +561,13 @@
       <c r="E4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="3" t="s">
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="B5" t="s">
         <v>8</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
       </c>
       <c r="C5" s="4">
         <v>46391</v>
@@ -580,16 +578,13 @@
       <c r="E5" s="5">
         <v>2906</v>
       </c>
-      <c r="F5" s="5">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
         <v>10</v>
-      </c>
-      <c r="B6" t="s">
-        <v>11</v>
       </c>
       <c r="C6" s="4">
         <v>46419</v>
@@ -600,19 +595,16 @@
       <c r="E6" s="5">
         <v>3995</v>
       </c>
-      <c r="F6" s="5">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" t="s">
         <v>12</v>
       </c>
-      <c r="B7" t="s">
-        <v>13</v>
-      </c>
       <c r="C7" s="4">
-        <v>46483</v>
+        <v>46490</v>
       </c>
       <c r="D7" s="5">
         <v>4976</v>
@@ -620,13 +612,10 @@
       <c r="E7" s="5">
         <v>3408</v>
       </c>
-      <c r="F7" s="5">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B8" s="7"/>
       <c r="C8" s="7"/>
@@ -636,17 +625,22 @@
       <c r="E8" s="8">
         <v>10309</v>
       </c>
-      <c r="F8" s="8">
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" s="10">
         <v>300</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="9" t="s">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="11" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
         <v>16</v>
       </c>
     </row>
@@ -819,7 +813,7 @@
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="9" t="s">
+      <c r="A12" s="11" t="s">
         <v>31</v>
       </c>
     </row>
@@ -849,10 +843,10 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="12" t="s">
         <v>35</v>
       </c>
     </row>
@@ -861,7 +855,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="5">
-        <v>4290230</v>
+        <v>5307260</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -869,7 +863,7 @@
         <v>21</v>
       </c>
       <c r="B6" s="5">
-        <v>4196710</v>
+        <v>5266345</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -877,7 +871,7 @@
         <v>22</v>
       </c>
       <c r="B7" s="5">
-        <v>4991630</v>
+        <v>6353515</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -885,7 +879,7 @@
         <v>23</v>
       </c>
       <c r="B8" s="5">
-        <v>4348680</v>
+        <v>5330640</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -893,11 +887,11 @@
         <v>24</v>
       </c>
       <c r="B9" s="8">
-        <v>17827250</v>
+        <v>22257760</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="9" t="s">
+      <c r="A11" s="11" t="s">
         <v>36</v>
       </c>
     </row>

</xml_diff>

<commit_message>
PAUSED (task175): stage 4 round 2 fix, waiting on round 3 readers
Ask A's primary re-sited from a meter set again at the same premise (reader D's
first install per premise kept all 20 cells) to one lot carried under two
premises: a stalled build's meter set again at a premise the cashier's counter
sets up (street type typed out, no parcel), the stub keeping the first set.
Measured on six routes including reader D's quoted path: 0 of 24 kept. The
call (293.225, printed 300), all 20 connection cells and the four fee quarters
are unchanged, asserted (Z1, Z2). The judge's advisory reading (a permit
issued counted as a home standing) lands at 279.3, 4.3 inside the bin, row SF11.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task175/golden/uep_2027_permit_forecast.xlsx
+++ b/task175/golden/uep_2027_permit_forecast.xlsx
@@ -77,7 +77,7 @@
     <t>New single-family connections, fiscal 2026</t>
   </si>
   <si>
-    <t>A premise's first meter install, at a premise with no account opened before it; quarter of the install date.</t>
+    <t>A lot's first meter install, at a lot with no account opened before it, premises placed on lots by parcel or service address; quarter of the install date.</t>
   </si>
   <si>
     <t>Phase</t>
@@ -116,7 +116,7 @@
     <t>All served areas</t>
   </si>
   <si>
-    <t>AMI head-end installs at premises already billed before the install are meter exchanges, and a second install at a premise is a meter set again, not connections. Phases as the program schedule groups the areas; premises are placed by parcel or service address.</t>
+    <t>AMI head-end installs at lots already billed before the install are meter exchanges, and a later install at a lot, on its stub or on a premise set up at the counter, is a meter set again, not a connection. Phases as the program schedule groups the areas.</t>
   </si>
   <si>
     <t>Water and sewer capacity fees received, fiscal 2026</t>

</xml_diff>

<commit_message>
PAUSED (task175): stage 4 round 4 restructure, waiting on round 5 readers and judge
The connection cells fell in three straight rounds to careful lot placement
(reader G kept all 20), so the ask layer is restructured: connections cut to the
four completed phases' fiscal 2026 totals, and the weight moved to capacity fees
by phase and quarter (20 cells), each cell carrying the drawer-day receipt
identity that held in 8 of 8 blind reads and a receipt covering several permits.
Builders' receipts now cover permits in one phase. The chart moves to the fees,
the prompt follows, and CONN_PIN files one connection per lot at its first meter
(judge pass 4 note). Measured on every recorded reader path: 0 of 24 on all but
reader G's (4 of 24), pair ceiling 37.7. The call is unchanged (293.225, Z1).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task175/golden/uep_2027_permit_forecast.xlsx
+++ b/task175/golden/uep_2027_permit_forecast.xlsx
@@ -77,12 +77,39 @@
     <t>New single-family connections, fiscal 2026</t>
   </si>
   <si>
-    <t>A lot's first meter install, at a lot with no account opened before it, premises placed on lots by parcel or service address; quarter of the install date.</t>
+    <t>A lot's first meter install, at a lot with no account opened before it, premises placed on lots by parcel or service address; October 2025 to September 2026.</t>
   </si>
   <si>
     <t>Phase</t>
   </si>
   <si>
+    <t>Connections</t>
+  </si>
+  <si>
+    <t>Phase 1</t>
+  </si>
+  <si>
+    <t>Phase 2</t>
+  </si>
+  <si>
+    <t>Phase 3</t>
+  </si>
+  <si>
+    <t>Phase 4</t>
+  </si>
+  <si>
+    <t>Phases 1 to 4</t>
+  </si>
+  <si>
+    <t>AMI head-end installs at lots already billed before the install are meter exchanges, and a later install at a lot, on its stub or on a premise set up at the counter, is a meter set again, not a connection. Phases as the program schedule groups the areas.</t>
+  </si>
+  <si>
+    <t>Water and sewer capacity fees received, fiscal 2026 (USD)</t>
+  </si>
+  <si>
+    <t>Cashiering receipts, fee code CAPWS, by receipt date; each payment (receipt number and payer) counted once, in the phase of its permits' lots.</t>
+  </si>
+  <si>
     <t>Q1 Oct-Dec 2025</t>
   </si>
   <si>
@@ -101,34 +128,7 @@
     <t>Core service area</t>
   </si>
   <si>
-    <t>Phase 1</t>
-  </si>
-  <si>
-    <t>Phase 2</t>
-  </si>
-  <si>
-    <t>Phase 3</t>
-  </si>
-  <si>
-    <t>Phase 4</t>
-  </si>
-  <si>
     <t>All served areas</t>
-  </si>
-  <si>
-    <t>AMI head-end installs at lots already billed before the install are meter exchanges, and a later install at a lot, on its stub or on a premise set up at the counter, is a meter set again, not a connection. Phases as the program schedule groups the areas.</t>
-  </si>
-  <si>
-    <t>Water and sewer capacity fees received, fiscal 2026</t>
-  </si>
-  <si>
-    <t>Cashiering receipts, fee code CAPWS, by receipt date; each payment (receipt number and payer) counted once.</t>
-  </si>
-  <si>
-    <t>Quarter</t>
-  </si>
-  <si>
-    <t>Fees received (USD)</t>
   </si>
   <si>
     <t>A builder's receipt covering several permits carries the receipt amount on each permit line; receipt numbers run by drawer and day.</t>
@@ -651,170 +651,74 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{743A5ADB-B7E5-5717-8BE6-8264584E5DC3}">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
-    <col min="2" max="2" width="13.7109375" customWidth="1"/>
-    <col min="3" max="3" width="13.7109375" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" customWidth="1"/>
-    <col min="5" max="5" width="13.7109375" customWidth="1"/>
-    <col min="6" max="6" width="12.7109375" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="3" t="s">
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="B5" s="5">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="B6" s="5">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>23</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="B7" s="5">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="B8" s="5">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="5">
-        <v>47</v>
-      </c>
-      <c r="C5" s="5">
-        <v>35</v>
-      </c>
-      <c r="D5" s="5">
-        <v>42</v>
-      </c>
-      <c r="E5" s="5">
-        <v>29</v>
-      </c>
-      <c r="F5" s="5">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="B9" s="8">
+        <v>1357</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="11" t="s">
         <v>26</v>
-      </c>
-      <c r="B6" s="5">
-        <v>52</v>
-      </c>
-      <c r="C6" s="5">
-        <v>37</v>
-      </c>
-      <c r="D6" s="5">
-        <v>56</v>
-      </c>
-      <c r="E6" s="5">
-        <v>61</v>
-      </c>
-      <c r="F6" s="5">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>27</v>
-      </c>
-      <c r="B7" s="5">
-        <v>71</v>
-      </c>
-      <c r="C7" s="5">
-        <v>61</v>
-      </c>
-      <c r="D7" s="5">
-        <v>97</v>
-      </c>
-      <c r="E7" s="5">
-        <v>64</v>
-      </c>
-      <c r="F7" s="5">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>28</v>
-      </c>
-      <c r="B8" s="5">
-        <v>107</v>
-      </c>
-      <c r="C8" s="5">
-        <v>97</v>
-      </c>
-      <c r="D8" s="5">
-        <v>130</v>
-      </c>
-      <c r="E8" s="5">
-        <v>128</v>
-      </c>
-      <c r="F8" s="5">
-        <v>462</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>29</v>
-      </c>
-      <c r="B9" s="5">
-        <v>98</v>
-      </c>
-      <c r="C9" s="5">
-        <v>101</v>
-      </c>
-      <c r="D9" s="5">
-        <v>96</v>
-      </c>
-      <c r="E9" s="5">
-        <v>101</v>
-      </c>
-      <c r="F9" s="5">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="B10" s="8">
-        <v>375</v>
-      </c>
-      <c r="C10" s="8">
-        <v>331</v>
-      </c>
-      <c r="D10" s="8">
-        <v>421</v>
-      </c>
-      <c r="E10" s="8">
-        <v>383</v>
-      </c>
-      <c r="F10" s="8">
-        <v>1510</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="11" t="s">
-        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -824,74 +728,169 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26C14DBA-7307-508B-9286-0011A0DF740E}">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
-    <col min="2" max="2" width="20.7109375" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" customWidth="1"/>
+    <col min="3" max="3" width="14.7109375" customWidth="1"/>
+    <col min="4" max="4" width="14.7109375" customWidth="1"/>
+    <col min="5" max="5" width="14.7109375" customWidth="1"/>
+    <col min="6" max="6" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="F4" s="3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="12" t="s">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>34</v>
       </c>
-      <c r="B4" s="12" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>20</v>
-      </c>
       <c r="B5" s="5">
-        <v>5307260</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+        <v>526050</v>
+      </c>
+      <c r="C5" s="5">
+        <v>578655</v>
+      </c>
+      <c r="D5" s="5">
+        <v>531895</v>
+      </c>
+      <c r="E5" s="5">
+        <v>420840</v>
+      </c>
+      <c r="F5" s="5">
+        <v>2057440</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>21</v>
       </c>
       <c r="B6" s="5">
-        <v>5266345</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+        <v>859215</v>
+      </c>
+      <c r="C6" s="5">
+        <v>672175</v>
+      </c>
+      <c r="D6" s="5">
+        <v>835835</v>
+      </c>
+      <c r="E6" s="5">
+        <v>841680</v>
+      </c>
+      <c r="F6" s="5">
+        <v>3208905</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>22</v>
       </c>
       <c r="B7" s="5">
-        <v>6353515</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+        <v>999495</v>
+      </c>
+      <c r="C7" s="5">
+        <v>941045</v>
+      </c>
+      <c r="D7" s="5">
+        <v>1467095</v>
+      </c>
+      <c r="E7" s="5">
+        <v>754005</v>
+      </c>
+      <c r="F7" s="5">
+        <v>4161640</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>23</v>
       </c>
       <c r="B8" s="5">
-        <v>5330640</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
+        <v>1467095</v>
+      </c>
+      <c r="C8" s="5">
+        <v>1776880</v>
+      </c>
+      <c r="D8" s="5">
+        <v>1940540</v>
+      </c>
+      <c r="E8" s="5">
+        <v>1876245</v>
+      </c>
+      <c r="F8" s="5">
+        <v>7060760</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="8">
-        <v>22257760</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="11" t="s">
+      <c r="B9" s="5">
+        <v>1472940</v>
+      </c>
+      <c r="C9" s="5">
+        <v>1332660</v>
+      </c>
+      <c r="D9" s="5">
+        <v>1601530</v>
+      </c>
+      <c r="E9" s="5">
+        <v>1379420</v>
+      </c>
+      <c r="F9" s="5">
+        <v>5786550</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" s="8">
+        <v>5324795</v>
+      </c>
+      <c r="C10" s="8">
+        <v>5301415</v>
+      </c>
+      <c r="D10" s="8">
+        <v>6376895</v>
+      </c>
+      <c r="E10" s="8">
+        <v>5272190</v>
+      </c>
+      <c r="F10" s="8">
+        <v>22275295</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="11" t="s">
         <v>36</v>
       </c>
     </row>

</xml_diff>